<commit_message>
Fixes to meta data and manual fix on miscoding
</commit_message>
<xml_diff>
--- a/data/metadata/main_deps 2021 09 01.xlsx
+++ b/data/metadata/main_deps 2021 09 01.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20373"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20382"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshua.wallace\Documents\R projects\mwmi-scraper\data\metadata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\mwmi.govuk.data\data\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01927F2F-483C-404D-A1D6-257F82667F35}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F425D7A6-2F3A-4C31-9644-90E5EECDE894}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8196" xr2:uid="{4236C203-4C4D-42BE-AA3F-1262EC2F12B0}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="Organisations">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1907,7 +1907,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="FTE cannot be greater than Headcount_x000a_" sqref="A198:A1048576 D1:E1 B2:B37 A1:A195" xr:uid="{2266A7B9-2E31-4A6B-9624-214B908CE8CA}"/>
+    <dataValidation operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="FTE cannot be greater than Headcount_x000a_" sqref="A198:A1048576 D1:E1 A1:A195 B2:B37" xr:uid="{2266A7B9-2E31-4A6B-9624-214B908CE8CA}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>